<commit_message>
recent updates in 5.23.2025
</commit_message>
<xml_diff>
--- a/01_macro_economic/CPI/inflation_comp.xlsx
+++ b/01_macro_economic/CPI/inflation_comp.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F852"/>
+  <dimension ref="A1:F921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20884,6 +20884,1662 @@
         <v>-3.6</v>
       </c>
     </row>
+    <row r="853">
+      <c r="A853" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Food_at_home</t>
+        </is>
+      </c>
+      <c r="C853" t="n">
+        <v>8.057</v>
+      </c>
+      <c r="D853" t="n">
+        <v>0.153083</v>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F853" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C854" t="n">
+        <v>6.292</v>
+      </c>
+      <c r="D854" t="n">
+        <v>-0.012584</v>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F854" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C855" t="n">
+        <v>35.417</v>
+      </c>
+      <c r="D855" t="n">
+        <v>1.487514</v>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F855" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C856" t="n">
+        <v>2.839</v>
+      </c>
+      <c r="D856" t="n">
+        <v>0.315129</v>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F856" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Core_goods</t>
+        </is>
+      </c>
+      <c r="C857" t="n">
+        <v>19.372</v>
+      </c>
+      <c r="D857" t="n">
+        <v>-0.019372</v>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F857" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C858" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="D858" t="n">
+        <v>0.208125</v>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F858" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Core_svcs</t>
+        </is>
+      </c>
+      <c r="C859" t="n">
+        <v>22.398</v>
+      </c>
+      <c r="D859" t="n">
+        <v>0.6841709999999996</v>
+      </c>
+      <c r="E859" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F859" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="C860" t="n">
+        <v>42.222</v>
+      </c>
+      <c r="D860" t="n">
+        <v>0.928884</v>
+      </c>
+      <c r="E860" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F860" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C861" t="n">
+        <v>13.681</v>
+      </c>
+      <c r="D861" t="n">
+        <v>0.355706</v>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F861" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C862" t="n">
+        <v>6.292</v>
+      </c>
+      <c r="D862" t="n">
+        <v>-0.012584</v>
+      </c>
+      <c r="E862" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F862" t="n">
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C863" t="n">
+        <v>35.417</v>
+      </c>
+      <c r="D863" t="n">
+        <v>1.487514</v>
+      </c>
+      <c r="E863" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F863" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Used cars/trucks</t>
+        </is>
+      </c>
+      <c r="C864" t="n">
+        <v>2.388</v>
+      </c>
+      <c r="D864" t="n">
+        <v>0.019104</v>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F864" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>New Car</t>
+        </is>
+      </c>
+      <c r="C865" t="n">
+        <v>4.376</v>
+      </c>
+      <c r="D865" t="n">
+        <v>-0.013128</v>
+      </c>
+      <c r="E865" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F865" t="n">
+        <v>-0.3</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Used Car</t>
+        </is>
+      </c>
+      <c r="C866" t="n">
+        <v>2.388</v>
+      </c>
+      <c r="D866" t="n">
+        <v>0.019104</v>
+      </c>
+      <c r="E866" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F866" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C867" t="n">
+        <v>2.839</v>
+      </c>
+      <c r="D867" t="n">
+        <v>0.315129</v>
+      </c>
+      <c r="E867" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F867" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Auto Parts</t>
+        </is>
+      </c>
+      <c r="C868" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="D868" t="n">
+        <v>0.004356</v>
+      </c>
+      <c r="E868" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F868" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Auto Repair</t>
+        </is>
+      </c>
+      <c r="C869" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="D869" t="n">
+        <v>0.059044</v>
+      </c>
+      <c r="E869" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F869" t="n">
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C870" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="D870" t="n">
+        <v>0.208125</v>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F870" t="n">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C871" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="D871" t="n">
+        <v>0.08900999999999999</v>
+      </c>
+      <c r="E871" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F871" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="C872" t="n">
+        <v>1.334</v>
+      </c>
+      <c r="D872" t="n">
+        <v>0.02668</v>
+      </c>
+      <c r="E872" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F872" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Airlines</t>
+        </is>
+      </c>
+      <c r="C873" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="D873" t="n">
+        <v>-0.006454</v>
+      </c>
+      <c r="E873" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F873" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+      <c r="C874" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="D874" t="n">
+        <v>0.01309</v>
+      </c>
+      <c r="E874" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F874" t="n">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Car Rental</t>
+        </is>
+      </c>
+      <c r="C875" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="D875" t="n">
+        <v>-0.008803999999999999</v>
+      </c>
+      <c r="E875" t="inlineStr">
+        <is>
+          <t>202502</t>
+        </is>
+      </c>
+      <c r="F875" t="n">
+        <v>-7.1</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Food_at_home</t>
+        </is>
+      </c>
+      <c r="C876" t="n">
+        <v>8.029999999999999</v>
+      </c>
+      <c r="D876" t="n">
+        <v>0.19272</v>
+      </c>
+      <c r="E876" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F876" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C877" t="n">
+        <v>6.329</v>
+      </c>
+      <c r="D877" t="n">
+        <v>-0.208857</v>
+      </c>
+      <c r="E877" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F877" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C878" t="n">
+        <v>35.389</v>
+      </c>
+      <c r="D878" t="n">
+        <v>1.41556</v>
+      </c>
+      <c r="E878" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F878" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C879" t="n">
+        <v>2.853</v>
+      </c>
+      <c r="D879" t="n">
+        <v>0.213975</v>
+      </c>
+      <c r="E879" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F879" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Core_goods</t>
+        </is>
+      </c>
+      <c r="C880" t="n">
+        <v>19.394</v>
+      </c>
+      <c r="D880" t="n">
+        <v>-0.019394</v>
+      </c>
+      <c r="E880" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F880" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C881" t="n">
+        <v>5.621</v>
+      </c>
+      <c r="D881" t="n">
+        <v>0.213598</v>
+      </c>
+      <c r="E881" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F881" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Core_svcs</t>
+        </is>
+      </c>
+      <c r="C882" t="n">
+        <v>22.38399999999999</v>
+      </c>
+      <c r="D882" t="n">
+        <v>0.6136269999999997</v>
+      </c>
+      <c r="E882" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F882" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="C883" t="n">
+        <v>42.253</v>
+      </c>
+      <c r="D883" t="n">
+        <v>0.7605540000000001</v>
+      </c>
+      <c r="E883" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F883" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C884" t="n">
+        <v>13.651</v>
+      </c>
+      <c r="D884" t="n">
+        <v>0.40953</v>
+      </c>
+      <c r="E884" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F884" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C885" t="n">
+        <v>6.329</v>
+      </c>
+      <c r="D885" t="n">
+        <v>-0.208857</v>
+      </c>
+      <c r="E885" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F885" t="n">
+        <v>-3.3</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C886" t="n">
+        <v>35.389</v>
+      </c>
+      <c r="D886" t="n">
+        <v>1.41556</v>
+      </c>
+      <c r="E886" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F886" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Used cars/trucks</t>
+        </is>
+      </c>
+      <c r="C887" t="n">
+        <v>2.378</v>
+      </c>
+      <c r="D887" t="n">
+        <v>0.014268</v>
+      </c>
+      <c r="E887" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F887" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>New Car</t>
+        </is>
+      </c>
+      <c r="C888" t="n">
+        <v>4.357</v>
+      </c>
+      <c r="D888" t="n">
+        <v>0</v>
+      </c>
+      <c r="E888" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F888" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Used Car</t>
+        </is>
+      </c>
+      <c r="C889" t="n">
+        <v>2.378</v>
+      </c>
+      <c r="D889" t="n">
+        <v>0.014268</v>
+      </c>
+      <c r="E889" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F889" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C890" t="n">
+        <v>2.853</v>
+      </c>
+      <c r="D890" t="n">
+        <v>0.213975</v>
+      </c>
+      <c r="E890" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F890" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Auto Parts</t>
+        </is>
+      </c>
+      <c r="C891" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D891" t="n">
+        <v>0.00432</v>
+      </c>
+      <c r="E891" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F891" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Auto Repair</t>
+        </is>
+      </c>
+      <c r="C892" t="n">
+        <v>1.016</v>
+      </c>
+      <c r="D892" t="n">
+        <v>0.04876800000000001</v>
+      </c>
+      <c r="E892" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F892" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C893" t="n">
+        <v>5.621</v>
+      </c>
+      <c r="D893" t="n">
+        <v>0.213598</v>
+      </c>
+      <c r="E893" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F893" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C894" t="n">
+        <v>2.075</v>
+      </c>
+      <c r="D894" t="n">
+        <v>0.1162</v>
+      </c>
+      <c r="E894" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F894" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="C895" t="n">
+        <v>1.366</v>
+      </c>
+      <c r="D895" t="n">
+        <v>-0.03415</v>
+      </c>
+      <c r="E895" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F895" t="n">
+        <v>-2.5</v>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Airlines</t>
+        </is>
+      </c>
+      <c r="C896" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="D896" t="n">
+        <v>-0.047164</v>
+      </c>
+      <c r="E896" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F896" t="n">
+        <v>-5.2</v>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+      <c r="C897" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="D897" t="n">
+        <v>0.01232</v>
+      </c>
+      <c r="E897" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F897" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Car Rental</t>
+        </is>
+      </c>
+      <c r="C898" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="D898" t="n">
+        <v>-0.010701</v>
+      </c>
+      <c r="E898" t="inlineStr">
+        <is>
+          <t>202503</t>
+        </is>
+      </c>
+      <c r="F898" t="n">
+        <v>-8.699999999999999</v>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Food_at_home</t>
+        </is>
+      </c>
+      <c r="C899" t="n">
+        <v>8.051</v>
+      </c>
+      <c r="D899" t="n">
+        <v>0.16102</v>
+      </c>
+      <c r="E899" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F899" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C900" t="n">
+        <v>6.312</v>
+      </c>
+      <c r="D900" t="n">
+        <v>-0.233544</v>
+      </c>
+      <c r="E900" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F900" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C901" t="n">
+        <v>35.426</v>
+      </c>
+      <c r="D901" t="n">
+        <v>1.41704</v>
+      </c>
+      <c r="E901" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F901" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C902" t="n">
+        <v>2.829</v>
+      </c>
+      <c r="D902" t="n">
+        <v>0.181056</v>
+      </c>
+      <c r="E902" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F902" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Core_goods</t>
+        </is>
+      </c>
+      <c r="C903" t="n">
+        <v>19.367</v>
+      </c>
+      <c r="D903" t="n">
+        <v>0.019367</v>
+      </c>
+      <c r="E903" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F903" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C904" t="n">
+        <v>5.629</v>
+      </c>
+      <c r="D904" t="n">
+        <v>0.219531</v>
+      </c>
+      <c r="E904" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F904" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Core_svcs</t>
+        </is>
+      </c>
+      <c r="C905" t="n">
+        <v>22.385</v>
+      </c>
+      <c r="D905" t="n">
+        <v>0.584944</v>
+      </c>
+      <c r="E905" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F905" t="n">
+        <v>-999</v>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Rest</t>
+        </is>
+      </c>
+      <c r="C906" t="n">
+        <v>42.201</v>
+      </c>
+      <c r="D906" t="n">
+        <v>0.759618</v>
+      </c>
+      <c r="E906" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F906" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="C907" t="n">
+        <v>13.681</v>
+      </c>
+      <c r="D907" t="n">
+        <v>0.383068</v>
+      </c>
+      <c r="E907" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F907" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C908" t="n">
+        <v>6.312</v>
+      </c>
+      <c r="D908" t="n">
+        <v>-0.233544</v>
+      </c>
+      <c r="E908" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F908" t="n">
+        <v>-3.7</v>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Shelter</t>
+        </is>
+      </c>
+      <c r="C909" t="n">
+        <v>35.426</v>
+      </c>
+      <c r="D909" t="n">
+        <v>1.41704</v>
+      </c>
+      <c r="E909" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F909" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Used cars/trucks</t>
+        </is>
+      </c>
+      <c r="C910" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="D910" t="n">
+        <v>0.0357</v>
+      </c>
+      <c r="E910" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F910" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>New Car</t>
+        </is>
+      </c>
+      <c r="C911" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="D911" t="n">
+        <v>0.01305</v>
+      </c>
+      <c r="E911" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F911" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Used Car</t>
+        </is>
+      </c>
+      <c r="C912" t="n">
+        <v>2.38</v>
+      </c>
+      <c r="D912" t="n">
+        <v>0.0357</v>
+      </c>
+      <c r="E912" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F912" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Auto Insurance</t>
+        </is>
+      </c>
+      <c r="C913" t="n">
+        <v>2.829</v>
+      </c>
+      <c r="D913" t="n">
+        <v>0.181056</v>
+      </c>
+      <c r="E913" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F913" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Auto Parts</t>
+        </is>
+      </c>
+      <c r="C914" t="n">
+        <v>0.358</v>
+      </c>
+      <c r="D914" t="n">
+        <v>0.004295999999999999</v>
+      </c>
+      <c r="E914" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F914" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="n">
+        <v>3000</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Auto Repair</t>
+        </is>
+      </c>
+      <c r="C915" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="D915" t="n">
+        <v>0.05723199999999999</v>
+      </c>
+      <c r="E915" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F915" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Dining</t>
+        </is>
+      </c>
+      <c r="C916" t="n">
+        <v>5.629</v>
+      </c>
+      <c r="D916" t="n">
+        <v>0.219531</v>
+      </c>
+      <c r="E916" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F916" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C917" t="n">
+        <v>2.078</v>
+      </c>
+      <c r="D917" t="n">
+        <v>0.105978</v>
+      </c>
+      <c r="E917" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F917" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Hotel</t>
+        </is>
+      </c>
+      <c r="C918" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="D918" t="n">
+        <v>-0.01925</v>
+      </c>
+      <c r="E918" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F918" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Airlines</t>
+        </is>
+      </c>
+      <c r="C919" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="D919" t="n">
+        <v>-0.068888</v>
+      </c>
+      <c r="E919" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F919" t="n">
+        <v>-7.9</v>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Beverage</t>
+        </is>
+      </c>
+      <c r="C920" t="n">
+        <v>0.385</v>
+      </c>
+      <c r="D920" t="n">
+        <v>0.01155</v>
+      </c>
+      <c r="E920" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F920" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="n">
+        <v>4000</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Car Rental</t>
+        </is>
+      </c>
+      <c r="C921" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="D921" t="n">
+        <v>-0.002667</v>
+      </c>
+      <c r="E921" t="inlineStr">
+        <is>
+          <t>202504</t>
+        </is>
+      </c>
+      <c r="F921" t="n">
+        <v>-2.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>